<commit_message>
Complete data preparation and proposal artifacts
</commit_message>
<xml_diff>
--- a/timeline/Master_Thesis_Timeline_2026_2027.xlsx
+++ b/timeline/Master_Thesis_Timeline_2026_2027.xlsx
@@ -1215,6 +1215,11 @@
   <mergeCells count="1">
     <mergeCell ref="A1:H1"/>
   </mergeCells>
+  <dataValidations count="1">
+    <dataValidation sqref="H4:H18" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="0" errorTitle="Invalid status" error="Select a status from the dropdown list." promptTitle="Task status" prompt="Choose the task status." type="list">
+      <formula1>"Pending,In Progress,Completed,CRITICAL"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>